<commit_message>
Complete runtime design calculations, construction reference and release packaging
</commit_message>
<xml_diff>
--- a/enterprise/runtime/publications/runtime-design-review-v1.0.0.xlsx
+++ b/enterprise/runtime/publications/runtime-design-review-v1.0.0.xlsx
@@ -19,13 +19,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Capacity!$A$5:$L$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cash requests'!$A$5:$J$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Enterprise!$A$5:$G$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Investment!$A$5:$H$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Investment!$A$5:$K$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Phases!$A$5:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Workforce!$A$5:$E$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Capacity!$A$1:$M$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Cash requests'!$A$1:$K$49</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">Enterprise!$A$1:$H$23</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">Investment!$A$1:$I$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">Investment!$A$1:$L$49</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">Phases!$A$1:$H$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Summary!$A$1:$D$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">Workforce!$A$1:$F$15</definedName>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="125">
   <si>
     <t>Runtime estate design review</t>
   </si>
@@ -82,7 +82,7 @@
     <t>Capacity — synthetic design / conditional forecast</t>
   </si>
   <si>
-    <t>No real operational evidence. Unknown funding/settlement remains explicit. Source identity b025486ae365b333d889</t>
+    <t>No real operational evidence. Unknown funding/settlement remains explicit. Source identity c85e35880c683be6f229</t>
   </si>
   <si>
     <t>scenario</t>
@@ -185,6 +185,15 @@
   </si>
   <si>
     <t>migration assumption</t>
+  </si>
+  <si>
+    <t>conditional plant additions</t>
+  </si>
+  <si>
+    <t>owned capacity kw</t>
+  </si>
+  <si>
+    <t>owned capacity sufficient</t>
   </si>
   <si>
     <t>Workforce — synthetic design / conditional forecast</t>
@@ -1228,19 +1237,19 @@
         <v>22</v>
       </c>
       <c r="F10" s="6">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G10" s="6">
         <v>22</v>
       </c>
       <c r="H10" s="5">
-        <v>195.6</v>
+        <v>198.8</v>
       </c>
       <c r="I10" s="5">
-        <v>121.95</v>
+        <v>123.95</v>
       </c>
       <c r="J10" s="5">
-        <v>7060000</v>
+        <v>7220000</v>
       </c>
       <c r="K10" s="5">
         <v>773.97</v>
@@ -1270,19 +1279,19 @@
         <v>4</v>
       </c>
       <c r="F11" s="6">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G11" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H11" s="5">
-        <v>50</v>
+        <v>53.2</v>
       </c>
       <c r="I11" s="5">
-        <v>31.05</v>
+        <v>33.05</v>
       </c>
       <c r="J11" s="5">
-        <v>1972000</v>
+        <v>2132000</v>
       </c>
       <c r="K11" s="5">
         <v>773.97</v>
@@ -1312,19 +1321,19 @@
         <v>7</v>
       </c>
       <c r="F12" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G12" s="6">
         <v>7</v>
       </c>
       <c r="H12" s="5">
-        <v>62.8</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="I12" s="5">
-        <v>39.05</v>
+        <v>40.05</v>
       </c>
       <c r="J12" s="5">
-        <v>2252000</v>
+        <v>2332000</v>
       </c>
       <c r="K12" s="5">
         <v>90</v>
@@ -1354,19 +1363,19 @@
         <v>2</v>
       </c>
       <c r="F13" s="6">
+        <v>5</v>
+      </c>
+      <c r="G13" s="6">
         <v>3</v>
       </c>
-      <c r="G13" s="6">
-        <v>2</v>
-      </c>
       <c r="H13" s="5">
-        <v>22</v>
+        <v>23.6</v>
       </c>
       <c r="I13" s="5">
-        <v>13.6</v>
+        <v>14.6</v>
       </c>
       <c r="J13" s="5">
-        <v>828000</v>
+        <v>908000</v>
       </c>
       <c r="K13" s="5">
         <v>90</v>
@@ -1396,19 +1405,19 @@
         <v>7</v>
       </c>
       <c r="F14" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G14" s="6">
         <v>7</v>
       </c>
       <c r="H14" s="5">
-        <v>64.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="I14" s="5">
-        <v>40.05</v>
+        <v>41.05</v>
       </c>
       <c r="J14" s="5">
-        <v>2332000</v>
+        <v>2412000</v>
       </c>
       <c r="K14" s="5">
         <v>186.62</v>
@@ -1438,19 +1447,19 @@
         <v>2</v>
       </c>
       <c r="F15" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G15" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="5">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="I15" s="5">
-        <v>14.6</v>
+        <v>15.6</v>
       </c>
       <c r="J15" s="5">
-        <v>908000</v>
+        <v>988000</v>
       </c>
       <c r="K15" s="5">
         <v>186.62</v>
@@ -1480,19 +1489,19 @@
         <v>6</v>
       </c>
       <c r="F16" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G16" s="6">
         <v>6</v>
       </c>
       <c r="H16" s="5">
-        <v>61.2</v>
+        <v>62.8</v>
       </c>
       <c r="I16" s="5">
-        <v>38.05</v>
+        <v>39.05</v>
       </c>
       <c r="J16" s="5">
-        <v>2292000</v>
+        <v>2372000</v>
       </c>
       <c r="K16" s="5">
         <v>464.38</v>
@@ -1522,19 +1531,19 @@
         <v>2</v>
       </c>
       <c r="F17" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G17" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17" s="5">
-        <v>28.4</v>
+        <v>30</v>
       </c>
       <c r="I17" s="5">
-        <v>17.6</v>
+        <v>18.6</v>
       </c>
       <c r="J17" s="5">
-        <v>1148000</v>
+        <v>1228000</v>
       </c>
       <c r="K17" s="5">
         <v>464.38</v>
@@ -1609,7 +1618,7 @@
         <v>7</v>
       </c>
       <c r="G19" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" s="5">
         <v>33.2</v>
@@ -1648,19 +1657,19 @@
         <v>36</v>
       </c>
       <c r="F20" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G20" s="6">
         <v>36</v>
       </c>
       <c r="H20" s="5">
-        <v>302</v>
+        <v>303.6</v>
       </c>
       <c r="I20" s="5">
-        <v>188.5</v>
+        <v>189.5</v>
       </c>
       <c r="J20" s="5">
-        <v>10716000</v>
+        <v>10796000</v>
       </c>
       <c r="K20" s="5">
         <v>466.56</v>
@@ -1690,19 +1699,19 @@
         <v>5</v>
       </c>
       <c r="F21" s="6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G21" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H21" s="5">
-        <v>53.2</v>
+        <v>54.8</v>
       </c>
       <c r="I21" s="5">
-        <v>33.05</v>
+        <v>34.05</v>
       </c>
       <c r="J21" s="5">
-        <v>2012000</v>
+        <v>2092000</v>
       </c>
       <c r="K21" s="5">
         <v>466.56</v>
@@ -1732,19 +1741,19 @@
         <v>105</v>
       </c>
       <c r="F22" s="6">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G22" s="6">
         <v>105</v>
       </c>
       <c r="H22" s="5">
-        <v>869.2</v>
+        <v>872.4</v>
       </c>
       <c r="I22" s="5">
-        <v>542.75</v>
+        <v>544.75</v>
       </c>
       <c r="J22" s="5">
-        <v>30716000</v>
+        <v>30876000</v>
       </c>
       <c r="K22" s="5">
         <v>1160.95</v>
@@ -1774,19 +1783,19 @@
         <v>12</v>
       </c>
       <c r="F23" s="6">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G23" s="6">
         <v>12</v>
       </c>
       <c r="H23" s="5">
-        <v>121.2</v>
+        <v>124.4</v>
       </c>
       <c r="I23" s="5">
-        <v>75.5</v>
+        <v>77.5</v>
       </c>
       <c r="J23" s="5">
-        <v>4556000</v>
+        <v>4716000</v>
       </c>
       <c r="K23" s="5">
         <v>1160.95</v>
@@ -1984,19 +1993,19 @@
         <v>22</v>
       </c>
       <c r="F28" s="6">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G28" s="6">
         <v>22</v>
       </c>
       <c r="H28" s="5">
-        <v>195.6</v>
+        <v>198.8</v>
       </c>
       <c r="I28" s="5">
-        <v>121.95</v>
+        <v>123.95</v>
       </c>
       <c r="J28" s="5">
-        <v>7060000</v>
+        <v>7220000</v>
       </c>
       <c r="K28" s="5">
         <v>773.97</v>
@@ -2026,19 +2035,19 @@
         <v>4</v>
       </c>
       <c r="F29" s="6">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G29" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H29" s="5">
-        <v>50</v>
+        <v>53.2</v>
       </c>
       <c r="I29" s="5">
-        <v>31.05</v>
+        <v>33.05</v>
       </c>
       <c r="J29" s="5">
-        <v>1972000</v>
+        <v>2132000</v>
       </c>
       <c r="K29" s="5">
         <v>773.97</v>
@@ -2235,25 +2244,25 @@
         <v>6425000</v>
       </c>
       <c r="D8" s="5">
-        <v>560000</v>
+        <v>720000</v>
       </c>
       <c r="E8" s="5">
-        <v>4668516.2</v>
+        <v>4672224.2</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
       </c>
       <c r="G8" s="5">
-        <v>11653516.2</v>
+        <v>11817224.2</v>
       </c>
       <c r="H8" s="5">
-        <v>11653516.2</v>
+        <v>11817224.2</v>
       </c>
       <c r="I8" s="5">
-        <v>9631005.119999999</v>
+        <v>9766300.99</v>
       </c>
       <c r="J8" s="5">
-        <v>11653516.2</v>
+        <v>11817224.2</v>
       </c>
       <c r="K8" s="5">
         <f>ROUND(G8-C8-D8-E8,2)</f>
@@ -2271,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="5">
-        <v>440000</v>
+        <v>280000</v>
       </c>
       <c r="E9" s="5">
         <v>4822359.14</v>
@@ -2280,16 +2289,16 @@
         <v>0</v>
       </c>
       <c r="G9" s="5">
-        <v>5262359.14</v>
+        <v>5102359.14</v>
       </c>
       <c r="H9" s="5">
-        <v>5262359.14</v>
+        <v>5102359.14</v>
       </c>
       <c r="I9" s="5">
-        <v>3953688.31</v>
+        <v>3833477.94</v>
       </c>
       <c r="J9" s="5">
-        <v>5262359.14</v>
+        <v>5102359.14</v>
       </c>
       <c r="K9" s="5">
         <f>ROUND(G9-C9-D9-E9,2)</f>
@@ -2307,25 +2316,25 @@
         <v>0</v>
       </c>
       <c r="D10" s="5">
-        <v>304000</v>
+        <v>464000</v>
       </c>
       <c r="E10" s="5">
-        <v>4979350.63</v>
+        <v>4983284.45</v>
       </c>
       <c r="F10" s="5">
         <v>0</v>
       </c>
       <c r="G10" s="5">
-        <v>5283350.63</v>
+        <v>5447284.45</v>
       </c>
       <c r="H10" s="5">
-        <v>5283350.63</v>
+        <v>5447284.45</v>
       </c>
       <c r="I10" s="5">
-        <v>3608599.57</v>
+        <v>3720568.57</v>
       </c>
       <c r="J10" s="5">
-        <v>5283350.63</v>
+        <v>5447284.45</v>
       </c>
       <c r="K10" s="5">
         <f>ROUND(G10-C10-D10-E10,2)</f>
@@ -2379,25 +2388,25 @@
         <v>0</v>
       </c>
       <c r="D12" s="5">
-        <v>280000</v>
+        <v>440000</v>
       </c>
       <c r="E12" s="5">
-        <v>5442998.42</v>
+        <v>5447171.81</v>
       </c>
       <c r="F12" s="5">
         <v>0</v>
       </c>
       <c r="G12" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="H12" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="I12" s="5">
-        <v>3230483.41</v>
+        <v>3323155.01</v>
       </c>
       <c r="J12" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="K12" s="5">
         <f>ROUND(G12-C12-D12-E12,2)</f>
@@ -2418,22 +2427,22 @@
         <v>440000</v>
       </c>
       <c r="E13" s="5">
-        <v>5633851.46</v>
+        <v>5763525.54</v>
       </c>
       <c r="F13" s="5">
         <v>0</v>
       </c>
       <c r="G13" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="H13" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="I13" s="5">
-        <v>3116846.18</v>
+        <v>3183389.49</v>
       </c>
       <c r="J13" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="K13" s="5">
         <f>ROUND(G13-C13-D13-E13,2)</f>
@@ -2454,22 +2463,22 @@
         <v>744000</v>
       </c>
       <c r="E14" s="5">
-        <v>5967178.62</v>
+        <v>5971606.16</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
       </c>
       <c r="G14" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="H14" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="I14" s="5">
-        <v>3130814.35</v>
+        <v>3132879.84</v>
       </c>
       <c r="J14" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="K14" s="5">
         <f>ROUND(G14-C14-D14-E14,2)</f>
@@ -2487,25 +2496,25 @@
         <v>0</v>
       </c>
       <c r="D15" s="5">
-        <v>8008000</v>
+        <v>8168000</v>
       </c>
       <c r="E15" s="5">
-        <v>6319304.3</v>
+        <v>6323864.67</v>
       </c>
       <c r="F15" s="5">
         <v>0</v>
       </c>
       <c r="G15" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="H15" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="I15" s="5">
-        <v>6076175.63</v>
+        <v>6145965.29</v>
       </c>
       <c r="J15" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="K15" s="5">
         <f>ROUND(G15-C15-D15-E15,2)</f>
@@ -2523,25 +2532,25 @@
         <v>0</v>
       </c>
       <c r="D16" s="5">
-        <v>1024000</v>
+        <v>1184000</v>
       </c>
       <c r="E16" s="5">
-        <v>6580996.94</v>
+        <v>6590391.31</v>
       </c>
       <c r="F16" s="5">
         <v>0</v>
       </c>
       <c r="G16" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="H16" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="I16" s="5">
-        <v>2932055.54</v>
+        <v>2997364.4</v>
       </c>
       <c r="J16" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="K16" s="5">
         <f>ROUND(G16-C16-D16-E16,2)</f>
@@ -2595,25 +2604,25 @@
         <v>4795000</v>
       </c>
       <c r="D18" s="5">
-        <v>3080000</v>
+        <v>3240000</v>
       </c>
       <c r="E18" s="5">
-        <v>4277450</v>
+        <v>4281050</v>
       </c>
       <c r="F18" s="5">
         <v>0</v>
       </c>
       <c r="G18" s="5">
-        <v>12152450</v>
+        <v>12316050</v>
       </c>
       <c r="H18" s="5">
-        <v>12152450</v>
+        <v>12316050</v>
       </c>
       <c r="I18" s="5">
-        <v>11047681.82</v>
+        <v>11196409.09</v>
       </c>
       <c r="J18" s="5">
-        <v>12152450</v>
+        <v>12316050</v>
       </c>
       <c r="K18" s="5">
         <f>ROUND(G18-C18-D18-E18,2)</f>
@@ -2631,7 +2640,7 @@
         <v>6425000</v>
       </c>
       <c r="D19" s="5">
-        <v>160000</v>
+        <v>0</v>
       </c>
       <c r="E19" s="5">
         <v>4414320.44</v>
@@ -2640,16 +2649,16 @@
         <v>0</v>
       </c>
       <c r="G19" s="5">
-        <v>10999320.44</v>
+        <v>10839320.44</v>
       </c>
       <c r="H19" s="5">
-        <v>10999320.44</v>
+        <v>10839320.44</v>
       </c>
       <c r="I19" s="5">
-        <v>9090347.470000001</v>
+        <v>8958116.07</v>
       </c>
       <c r="J19" s="5">
-        <v>10999320.44</v>
+        <v>10839320.44</v>
       </c>
       <c r="K19" s="5">
         <f>ROUND(G19-C19-D19-E19,2)</f>
@@ -2739,25 +2748,25 @@
         <v>0</v>
       </c>
       <c r="D22" s="5">
-        <v>3240000</v>
+        <v>3400000</v>
       </c>
       <c r="E22" s="5">
-        <v>4846742.37</v>
+        <v>4850794.2</v>
       </c>
       <c r="F22" s="5">
         <v>0</v>
       </c>
       <c r="G22" s="5">
-        <v>8086742.37</v>
+        <v>8250794.2</v>
       </c>
       <c r="H22" s="5">
-        <v>8086742.37</v>
+        <v>8250794.2</v>
       </c>
       <c r="I22" s="5">
-        <v>5021230.77</v>
+        <v>5123094.05</v>
       </c>
       <c r="J22" s="5">
-        <v>8086742.37</v>
+        <v>8250794.2</v>
       </c>
       <c r="K22" s="5">
         <f>ROUND(G22-C22-D22-E22,2)</f>
@@ -2775,7 +2784,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="5">
-        <v>160000</v>
+        <v>0</v>
       </c>
       <c r="E23" s="5">
         <v>5007612.99</v>
@@ -2784,16 +2793,16 @@
         <v>0</v>
       </c>
       <c r="G23" s="5">
-        <v>5167612.99</v>
+        <v>5007612.99</v>
       </c>
       <c r="H23" s="5">
-        <v>5167612.99</v>
+        <v>5007612.99</v>
       </c>
       <c r="I23" s="5">
-        <v>2916982.81</v>
+        <v>2826666.98</v>
       </c>
       <c r="J23" s="5">
-        <v>5167612.99</v>
+        <v>5007612.99</v>
       </c>
       <c r="K23" s="5">
         <f>ROUND(G23-C23-D23-E23,2)</f>
@@ -2814,22 +2823,22 @@
         <v>0</v>
       </c>
       <c r="E24" s="5">
-        <v>5171800.07</v>
+        <v>5176098.66</v>
       </c>
       <c r="F24" s="5">
         <v>0</v>
       </c>
       <c r="G24" s="5">
-        <v>5171800.07</v>
+        <v>5176098.66</v>
       </c>
       <c r="H24" s="5">
-        <v>5171800.07</v>
+        <v>5176098.66</v>
       </c>
       <c r="I24" s="5">
-        <v>2653951.19</v>
+        <v>2656157.05</v>
       </c>
       <c r="J24" s="5">
-        <v>5171800.07</v>
+        <v>5176098.66</v>
       </c>
       <c r="K24" s="5">
         <f>ROUND(G24-C24-D24-E24,2)</f>
@@ -2847,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="5">
-        <v>160000</v>
+        <v>0</v>
       </c>
       <c r="E25" s="5">
         <v>5348635.21</v>
@@ -2856,16 +2865,16 @@
         <v>0</v>
       </c>
       <c r="G25" s="5">
-        <v>5508635.21</v>
+        <v>5348635.21</v>
       </c>
       <c r="H25" s="5">
-        <v>5508635.21</v>
+        <v>5348635.21</v>
       </c>
       <c r="I25" s="5">
-        <v>2569818.98</v>
+        <v>2495177.8</v>
       </c>
       <c r="J25" s="5">
-        <v>5508635.21</v>
+        <v>5348635.21</v>
       </c>
       <c r="K25" s="5">
         <f>ROUND(G25-C25-D25-E25,2)</f>
@@ -2883,29 +2892,29 @@
         <v>0</v>
       </c>
       <c r="D26" s="5">
-        <v>3280000</v>
+        <v>3440000</v>
       </c>
       <c r="E26" s="5">
-        <v>5530416.41</v>
+        <v>5534976.78</v>
       </c>
       <c r="F26" s="5">
         <v>0</v>
       </c>
       <c r="G26" s="5">
-        <v>8810416.41</v>
+        <v>8974976.779999999</v>
       </c>
       <c r="H26" s="5">
-        <v>8810416.41</v>
+        <v>8974976.779999999</v>
       </c>
       <c r="I26" s="5">
-        <v>3736476.61</v>
+        <v>3806266.28</v>
       </c>
       <c r="J26" s="5">
-        <v>8810416.41</v>
+        <v>8974976.779999999</v>
       </c>
       <c r="K26" s="5">
         <f>ROUND(G26-C26-D26-E26,2)</f>
-        <v>0.0</v>
+        <v>-0.0</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="28" customHeight="1">
@@ -2922,22 +2931,22 @@
         <v>160000</v>
       </c>
       <c r="E27" s="5">
-        <v>5727384.33</v>
+        <v>5732081.51</v>
       </c>
       <c r="F27" s="5">
         <v>0</v>
       </c>
       <c r="G27" s="5">
-        <v>5887384.33</v>
+        <v>5892081.51</v>
       </c>
       <c r="H27" s="5">
-        <v>5887384.33</v>
+        <v>5892081.51</v>
       </c>
       <c r="I27" s="5">
-        <v>2269841.52</v>
+        <v>2271652.49</v>
       </c>
       <c r="J27" s="5">
-        <v>5887384.33</v>
+        <v>5892081.51</v>
       </c>
       <c r="K27" s="5">
         <f>ROUND(G27-C27-D27-E27,2)</f>
@@ -3027,25 +3036,25 @@
         <v>6425000</v>
       </c>
       <c r="D30" s="5">
-        <v>1144000</v>
+        <v>1304000</v>
       </c>
       <c r="E30" s="5">
-        <v>4912718.9</v>
+        <v>4916426.9</v>
       </c>
       <c r="F30" s="5">
         <v>0</v>
       </c>
       <c r="G30" s="5">
-        <v>12481718.9</v>
+        <v>12645426.9</v>
       </c>
       <c r="H30" s="5">
-        <v>12481718.9</v>
+        <v>12645426.9</v>
       </c>
       <c r="I30" s="5">
-        <v>10315470.17</v>
+        <v>10450766.03</v>
       </c>
       <c r="J30" s="5">
-        <v>12481718.9</v>
+        <v>12645426.9</v>
       </c>
       <c r="K30" s="5">
         <f>ROUND(G30-C30-D30-E30,2)</f>
@@ -3063,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="5">
-        <v>1560000</v>
+        <v>1400000</v>
       </c>
       <c r="E31" s="5">
         <v>5209362.73</v>
@@ -3072,16 +3081,16 @@
         <v>0</v>
       </c>
       <c r="G31" s="5">
-        <v>6769362.73</v>
+        <v>6609362.73</v>
       </c>
       <c r="H31" s="5">
-        <v>6769362.73</v>
+        <v>6609362.73</v>
       </c>
       <c r="I31" s="5">
-        <v>5085922.41</v>
+        <v>4965712.04</v>
       </c>
       <c r="J31" s="5">
-        <v>6769362.73</v>
+        <v>6609362.73</v>
       </c>
       <c r="K31" s="5">
         <f>ROUND(G31-C31-D31-E31,2)</f>
@@ -3099,25 +3108,25 @@
         <v>0</v>
       </c>
       <c r="D32" s="5">
-        <v>1704000</v>
+        <v>1864000</v>
       </c>
       <c r="E32" s="5">
-        <v>5615367.57</v>
+        <v>5619301.39</v>
       </c>
       <c r="F32" s="5">
         <v>0</v>
       </c>
       <c r="G32" s="5">
-        <v>7319367.57</v>
+        <v>7483301.39</v>
       </c>
       <c r="H32" s="5">
-        <v>7319367.57</v>
+        <v>7483301.39</v>
       </c>
       <c r="I32" s="5">
-        <v>4999226.54</v>
+        <v>5111195.54</v>
       </c>
       <c r="J32" s="5">
-        <v>7319367.57</v>
+        <v>7483301.39</v>
       </c>
       <c r="K32" s="5">
         <f>ROUND(G32-C32-D32-E32,2)</f>
@@ -3135,25 +3144,25 @@
         <v>0</v>
       </c>
       <c r="D33" s="5">
-        <v>12728000</v>
+        <v>12888000</v>
       </c>
       <c r="E33" s="5">
-        <v>6185517.47</v>
+        <v>6189569.31</v>
       </c>
       <c r="F33" s="5">
         <v>0</v>
       </c>
       <c r="G33" s="5">
-        <v>18913517.47</v>
+        <v>19077569.31</v>
       </c>
       <c r="H33" s="5">
-        <v>18913517.47</v>
+        <v>19077569.31</v>
       </c>
       <c r="I33" s="5">
-        <v>11743806.29</v>
+        <v>11845669.57</v>
       </c>
       <c r="J33" s="5">
-        <v>18913517.47</v>
+        <v>19077569.31</v>
       </c>
       <c r="K33" s="5">
         <f>ROUND(G33-C33-D33-E33,2)</f>
@@ -3174,26 +3183,26 @@
         <v>2704000</v>
       </c>
       <c r="E34" s="5">
-        <v>6667803.73</v>
+        <v>6671977.12</v>
       </c>
       <c r="F34" s="5">
         <v>0</v>
       </c>
       <c r="G34" s="5">
-        <v>9371803.73</v>
+        <v>9375977.119999999</v>
       </c>
       <c r="H34" s="5">
-        <v>9371803.73</v>
+        <v>9375977.119999999</v>
       </c>
       <c r="I34" s="5">
-        <v>5290138.88</v>
+        <v>5292494.65</v>
       </c>
       <c r="J34" s="5">
-        <v>9371803.73</v>
+        <v>9375977.119999999</v>
       </c>
       <c r="K34" s="5">
         <f>ROUND(G34-C34-D34-E34,2)</f>
-        <v>0.0</v>
+        <v>-0.0</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="28" customHeight="1">
@@ -3207,25 +3216,25 @@
         <v>0</v>
       </c>
       <c r="D35" s="5">
-        <v>3544000</v>
+        <v>3704000</v>
       </c>
       <c r="E35" s="5">
-        <v>7430029.64</v>
+        <v>7438626.82</v>
       </c>
       <c r="F35" s="5">
         <v>0</v>
       </c>
       <c r="G35" s="5">
-        <v>10974029.64</v>
+        <v>11142626.82</v>
       </c>
       <c r="H35" s="5">
-        <v>10974029.64</v>
+        <v>11142626.82</v>
       </c>
       <c r="I35" s="5">
-        <v>5631412.4</v>
+        <v>5717929.41</v>
       </c>
       <c r="J35" s="5">
-        <v>10974029.64</v>
+        <v>11142626.82</v>
       </c>
       <c r="K35" s="5">
         <f>ROUND(G35-C35-D35-E35,2)</f>
@@ -3243,25 +3252,25 @@
         <v>0</v>
       </c>
       <c r="D36" s="5">
-        <v>4240000</v>
+        <v>4080000</v>
       </c>
       <c r="E36" s="5">
-        <v>8243602.75</v>
+        <v>8248030.3</v>
       </c>
       <c r="F36" s="5">
         <v>0</v>
       </c>
       <c r="G36" s="5">
-        <v>12483602.75</v>
+        <v>12328030.3</v>
       </c>
       <c r="H36" s="5">
-        <v>12483602.75</v>
+        <v>12328030.3</v>
       </c>
       <c r="I36" s="5">
-        <v>5823692.82</v>
+        <v>5751117.12</v>
       </c>
       <c r="J36" s="5">
-        <v>12483602.75</v>
+        <v>12328030.3</v>
       </c>
       <c r="K36" s="5">
         <f>ROUND(G36-C36-D36-E36,2)</f>
@@ -3279,25 +3288,25 @@
         <v>0</v>
       </c>
       <c r="D37" s="5">
-        <v>28744000</v>
+        <v>29064000</v>
       </c>
       <c r="E37" s="5">
-        <v>9394502.539999999</v>
+        <v>9403623.289999999</v>
       </c>
       <c r="F37" s="5">
         <v>0</v>
       </c>
       <c r="G37" s="5">
-        <v>38138502.54</v>
+        <v>38467623.29</v>
       </c>
       <c r="H37" s="5">
-        <v>38138502.54</v>
+        <v>38467623.29</v>
       </c>
       <c r="I37" s="5">
-        <v>16174448.1</v>
+        <v>16314027.42</v>
       </c>
       <c r="J37" s="5">
-        <v>38138502.54</v>
+        <v>38467623.29</v>
       </c>
       <c r="K37" s="5">
         <f>ROUND(G37-C37-D37-E37,2)</f>
@@ -3318,26 +3327,26 @@
         <v>6528000</v>
       </c>
       <c r="E38" s="5">
-        <v>10620603.13</v>
+        <v>10629997.5</v>
       </c>
       <c r="F38" s="5">
         <v>0</v>
       </c>
       <c r="G38" s="5">
-        <v>17148603.13</v>
+        <v>17157997.5</v>
       </c>
       <c r="H38" s="5">
-        <v>17148603.13</v>
+        <v>17157997.5</v>
       </c>
       <c r="I38" s="5">
-        <v>6611528.86</v>
+        <v>6615150.8</v>
       </c>
       <c r="J38" s="5">
-        <v>17148603.13</v>
+        <v>17157997.5</v>
       </c>
       <c r="K38" s="5">
         <f>ROUND(G38-C38-D38-E38,2)</f>
-        <v>-0.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="28" customHeight="1">
@@ -3423,25 +3432,25 @@
         <v>0</v>
       </c>
       <c r="D41" s="5">
-        <v>560000</v>
+        <v>720000</v>
       </c>
       <c r="E41" s="5">
-        <v>4668516.2</v>
+        <v>4672224.2</v>
       </c>
       <c r="F41" s="5">
         <v>0</v>
       </c>
       <c r="G41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="H41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="I41" s="5">
-        <v>4321087.77</v>
+        <v>4456383.64</v>
       </c>
       <c r="J41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="K41" s="5">
         <f>ROUND(G41-C41-D41-E41,2)</f>
@@ -3459,7 +3468,7 @@
         <v>4375000</v>
       </c>
       <c r="D42" s="5">
-        <v>440000</v>
+        <v>280000</v>
       </c>
       <c r="E42" s="5">
         <v>4822359.14</v>
@@ -3468,16 +3477,16 @@
         <v>0</v>
       </c>
       <c r="G42" s="5">
-        <v>9637359.140000001</v>
+        <v>9477359.140000001</v>
       </c>
       <c r="H42" s="5">
-        <v>9637359.140000001</v>
+        <v>9477359.140000001</v>
       </c>
       <c r="I42" s="5">
-        <v>7240690.57</v>
+        <v>7120480.2</v>
       </c>
       <c r="J42" s="5">
-        <v>9637359.140000001</v>
+        <v>9477359.140000001</v>
       </c>
       <c r="K42" s="5">
         <f>ROUND(G42-C42-D42-E42,2)</f>
@@ -3495,29 +3504,29 @@
         <v>6425000</v>
       </c>
       <c r="D43" s="5">
-        <v>304000</v>
+        <v>464000</v>
       </c>
       <c r="E43" s="5">
-        <v>4979350.63</v>
+        <v>4983284.45</v>
       </c>
       <c r="F43" s="5">
         <v>0</v>
       </c>
       <c r="G43" s="5">
-        <v>11708350.63</v>
+        <v>11872284.45</v>
       </c>
       <c r="H43" s="5">
-        <v>11708350.63</v>
+        <v>11872284.45</v>
       </c>
       <c r="I43" s="5">
-        <v>7996961.02</v>
+        <v>8108930.02</v>
       </c>
       <c r="J43" s="5">
-        <v>11708350.63</v>
+        <v>11872284.45</v>
       </c>
       <c r="K43" s="5">
         <f>ROUND(G43-C43-D43-E43,2)</f>
-        <v>0.0</v>
+        <v>-0.0</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="28" customHeight="1">
@@ -3567,25 +3576,25 @@
         <v>0</v>
       </c>
       <c r="D45" s="5">
-        <v>280000</v>
+        <v>440000</v>
       </c>
       <c r="E45" s="5">
-        <v>5442998.42</v>
+        <v>5447171.81</v>
       </c>
       <c r="F45" s="5">
         <v>0</v>
       </c>
       <c r="G45" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="H45" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="I45" s="5">
-        <v>3230483.41</v>
+        <v>3323155.01</v>
       </c>
       <c r="J45" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="K45" s="5">
         <f>ROUND(G45-C45-D45-E45,2)</f>
@@ -3606,22 +3615,22 @@
         <v>440000</v>
       </c>
       <c r="E46" s="5">
-        <v>5633851.46</v>
+        <v>5763525.54</v>
       </c>
       <c r="F46" s="5">
         <v>0</v>
       </c>
       <c r="G46" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="H46" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="I46" s="5">
-        <v>3116846.18</v>
+        <v>3183389.49</v>
       </c>
       <c r="J46" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="K46" s="5">
         <f>ROUND(G46-C46-D46-E46,2)</f>
@@ -3642,22 +3651,22 @@
         <v>744000</v>
       </c>
       <c r="E47" s="5">
-        <v>5967178.62</v>
+        <v>5971606.16</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
       </c>
       <c r="G47" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="H47" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="I47" s="5">
-        <v>3130814.35</v>
+        <v>3132879.84</v>
       </c>
       <c r="J47" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="K47" s="5">
         <f>ROUND(G47-C47-D47-E47,2)</f>
@@ -3675,25 +3684,25 @@
         <v>0</v>
       </c>
       <c r="D48" s="5">
-        <v>8008000</v>
+        <v>8168000</v>
       </c>
       <c r="E48" s="5">
-        <v>6319304.3</v>
+        <v>6323864.67</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
       </c>
       <c r="G48" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="H48" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="I48" s="5">
-        <v>6076175.63</v>
+        <v>6145965.29</v>
       </c>
       <c r="J48" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="K48" s="5">
         <f>ROUND(G48-C48-D48-E48,2)</f>
@@ -3711,25 +3720,25 @@
         <v>0</v>
       </c>
       <c r="D49" s="5">
-        <v>1024000</v>
+        <v>1184000</v>
       </c>
       <c r="E49" s="5">
-        <v>6580996.94</v>
+        <v>6590391.31</v>
       </c>
       <c r="F49" s="5">
         <v>0</v>
       </c>
       <c r="G49" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="H49" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="I49" s="5">
-        <v>2932055.54</v>
+        <v>2997364.4</v>
       </c>
       <c r="J49" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="K49" s="5">
         <f>ROUND(G49-C49-D49-E49,2)</f>
@@ -3755,14 +3764,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="9" width="17.7109375" customWidth="1"/>
+    <col min="2" max="12" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
@@ -3773,8 +3782,11 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="25" customHeight="1">
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:12" ht="25" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -3785,8 +3797,11 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" ht="18" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3795,8 +3810,11 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-    </row>
-    <row r="5" spans="1:9" ht="36" customHeight="1">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="36" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -3822,10 +3840,19 @@
         <v>47</v>
       </c>
       <c r="I5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="28" customHeight="1">
+    <row r="6" spans="1:12" ht="28" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
@@ -3851,11 +3878,20 @@
         <v>2029</v>
       </c>
       <c r="I6" s="5">
+        <v>0</v>
+      </c>
+      <c r="J6" s="5">
+        <v>250</v>
+      </c>
+      <c r="K6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="5">
         <f>ROUND(F6-D6+E6,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="28" customHeight="1">
+    <row r="7" spans="1:12" ht="28" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
@@ -3881,11 +3917,20 @@
         <v>2029</v>
       </c>
       <c r="I7" s="5">
+        <v>0</v>
+      </c>
+      <c r="J7" s="5">
+        <v>250</v>
+      </c>
+      <c r="K7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="5">
         <f>ROUND(F7-D7+E7,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28" customHeight="1">
+    <row r="8" spans="1:12" ht="28" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
@@ -3893,16 +3938,16 @@
         <v>2028</v>
       </c>
       <c r="C8" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="D8" s="5">
-        <v>11653516.2</v>
+        <v>11817224.2</v>
       </c>
       <c r="E8" s="5">
         <v>0</v>
       </c>
       <c r="F8" s="5">
-        <v>11653516.2</v>
+        <v>11817224.2</v>
       </c>
       <c r="G8" s="5">
         <v>5309917.36</v>
@@ -3911,11 +3956,20 @@
         <v>2029</v>
       </c>
       <c r="I8" s="5">
+        <v>0</v>
+      </c>
+      <c r="J8" s="5">
+        <v>250</v>
+      </c>
+      <c r="K8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5">
         <f>ROUND(F8-D8+E8,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="28" customHeight="1">
+    <row r="9" spans="1:12" ht="28" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>3</v>
       </c>
@@ -3923,29 +3977,38 @@
         <v>2029</v>
       </c>
       <c r="C9" s="5">
-        <v>5262359.14</v>
+        <v>5102359.14</v>
       </c>
       <c r="D9" s="5">
-        <v>6782170.14</v>
+        <v>6704281.44</v>
       </c>
       <c r="E9" s="5">
         <v>0</v>
       </c>
       <c r="F9" s="5">
-        <v>6782170.14</v>
+        <v>6704281.44</v>
       </c>
       <c r="G9" s="5">
-        <v>1141856.5</v>
+        <v>1203547.94</v>
       </c>
       <c r="H9" s="6">
         <v>2029</v>
       </c>
       <c r="I9" s="5">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5">
+        <v>250</v>
+      </c>
+      <c r="K9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="5">
         <f>ROUND(F9-D9+E9,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="28" customHeight="1">
+    <row r="10" spans="1:12" ht="28" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>3</v>
       </c>
@@ -3953,29 +4016,38 @@
         <v>2030</v>
       </c>
       <c r="C10" s="5">
-        <v>5283350.63</v>
+        <v>5447284.45</v>
       </c>
       <c r="D10" s="5">
-        <v>6066273.32</v>
+        <v>6357666.57</v>
       </c>
       <c r="E10" s="5">
         <v>0</v>
       </c>
       <c r="F10" s="5">
-        <v>6066273.32</v>
+        <v>6357666.57</v>
       </c>
       <c r="G10" s="5">
-        <v>534746.73</v>
+        <v>621803.23</v>
       </c>
       <c r="H10" s="6">
         <v>2029</v>
       </c>
       <c r="I10" s="5">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5">
+        <v>250</v>
+      </c>
+      <c r="K10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" s="5">
         <f>ROUND(F10-D10+E10,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="28" customHeight="1">
+    <row r="11" spans="1:12" ht="28" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>3</v>
       </c>
@@ -3986,26 +4058,35 @@
         <v>11370189.81</v>
       </c>
       <c r="D11" s="5">
-        <v>12026869.06</v>
+        <v>12198282.69</v>
       </c>
       <c r="E11" s="5">
         <v>0</v>
       </c>
       <c r="F11" s="5">
-        <v>12026869.06</v>
+        <v>12198282.69</v>
       </c>
       <c r="G11" s="5">
-        <v>407746.15</v>
+        <v>514180.53</v>
       </c>
       <c r="H11" s="6">
         <v>2029</v>
       </c>
       <c r="I11" s="5">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5">
+        <v>250</v>
+      </c>
+      <c r="K11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="5">
         <f>ROUND(F11-D11+E11,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="28" customHeight="1">
+    <row r="12" spans="1:12" ht="28" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>3</v>
       </c>
@@ -4013,29 +4094,38 @@
         <v>2032</v>
       </c>
       <c r="C12" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="D12" s="5">
-        <v>6366026.75</v>
+        <v>6750709.55</v>
       </c>
       <c r="E12" s="5">
         <v>0</v>
       </c>
       <c r="F12" s="5">
-        <v>6366026.75</v>
+        <v>6750709.55</v>
       </c>
       <c r="G12" s="5">
-        <v>362972.73</v>
+        <v>487444.54</v>
       </c>
       <c r="H12" s="6">
         <v>2029</v>
       </c>
       <c r="I12" s="5">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5">
+        <v>250</v>
+      </c>
+      <c r="K12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="5">
         <f>ROUND(F12-D12+E12,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="28" customHeight="1">
+    <row r="13" spans="1:12" ht="28" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
@@ -4043,29 +4133,38 @@
         <v>2033</v>
       </c>
       <c r="C13" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="D13" s="5">
-        <v>6704114.95</v>
+        <v>6978514.05</v>
       </c>
       <c r="E13" s="5">
         <v>0</v>
       </c>
       <c r="F13" s="5">
-        <v>6704114.95</v>
+        <v>6978514.05</v>
       </c>
       <c r="G13" s="5">
-        <v>323424.83</v>
+        <v>397691.65</v>
       </c>
       <c r="H13" s="6">
         <v>2029</v>
       </c>
       <c r="I13" s="5">
+        <v>0</v>
+      </c>
+      <c r="J13" s="5">
+        <v>250</v>
+      </c>
+      <c r="K13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="5">
         <f>ROUND(F13-D13+E13,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="28" customHeight="1">
+    <row r="14" spans="1:12" ht="28" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>3</v>
       </c>
@@ -4073,29 +4172,38 @@
         <v>2034</v>
       </c>
       <c r="C14" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="D14" s="5">
-        <v>7206504.41</v>
+        <v>8034465.18</v>
       </c>
       <c r="E14" s="5">
         <v>0</v>
       </c>
       <c r="F14" s="5">
-        <v>7206504.41</v>
+        <v>8034465.18</v>
       </c>
       <c r="G14" s="5">
-        <v>231073.14</v>
+        <v>615257.47</v>
       </c>
       <c r="H14" s="6">
         <v>2029</v>
       </c>
       <c r="I14" s="5">
+        <v>500000</v>
+      </c>
+      <c r="J14" s="5">
+        <v>250</v>
+      </c>
+      <c r="K14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="5">
         <f>ROUND(F14-D14+E14,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="28" customHeight="1">
+    <row r="15" spans="1:12" ht="28" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>3</v>
       </c>
@@ -4103,29 +4211,38 @@
         <v>2035</v>
       </c>
       <c r="C15" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="D15" s="5">
-        <v>14671645.95</v>
+        <v>15213863.77</v>
       </c>
       <c r="E15" s="5">
         <v>0</v>
       </c>
       <c r="F15" s="5">
-        <v>14671645.95</v>
+        <v>15213863.77</v>
       </c>
       <c r="G15" s="5">
-        <v>146034.47</v>
+        <v>306198.1</v>
       </c>
       <c r="H15" s="6">
         <v>2029</v>
       </c>
       <c r="I15" s="5">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5">
+        <v>250</v>
+      </c>
+      <c r="K15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="5">
         <f>ROUND(F15-D15+E15,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="28" customHeight="1">
+    <row r="16" spans="1:12" ht="28" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>3</v>
       </c>
@@ -4133,29 +4250,38 @@
         <v>2036</v>
       </c>
       <c r="C16" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="D16" s="5">
-        <v>8184868.53</v>
+        <v>8792810.789999999</v>
       </c>
       <c r="E16" s="5">
         <v>0</v>
       </c>
       <c r="F16" s="5">
-        <v>8184868.53</v>
+        <v>8792810.789999999</v>
       </c>
       <c r="G16" s="5">
-        <v>223565.6</v>
+        <v>392644.8</v>
       </c>
       <c r="H16" s="6">
         <v>2029</v>
       </c>
       <c r="I16" s="5">
+        <v>0</v>
+      </c>
+      <c r="J16" s="5">
+        <v>250</v>
+      </c>
+      <c r="K16" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="5">
         <f>ROUND(F16-D16+E16,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28" customHeight="1">
+    <row r="17" spans="1:12" ht="28" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
@@ -4181,11 +4307,20 @@
         <v>2029</v>
       </c>
       <c r="I17" s="5">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5">
+        <v>250</v>
+      </c>
+      <c r="K17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="5">
         <f>ROUND(F17-D17+E17,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="28" customHeight="1">
+    <row r="18" spans="1:12" ht="28" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>29</v>
       </c>
@@ -4193,16 +4328,16 @@
         <v>2027</v>
       </c>
       <c r="C18" s="5">
-        <v>7357450</v>
+        <v>7521050</v>
       </c>
       <c r="D18" s="5">
-        <v>12152450</v>
+        <v>12316050</v>
       </c>
       <c r="E18" s="5">
         <v>0</v>
       </c>
       <c r="F18" s="5">
-        <v>12152450</v>
+        <v>12316050</v>
       </c>
       <c r="G18" s="5">
         <v>4359090.91</v>
@@ -4211,11 +4346,20 @@
         <v>2029</v>
       </c>
       <c r="I18" s="5">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5">
+        <v>250</v>
+      </c>
+      <c r="K18" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="5">
         <f>ROUND(F18-D18+E18,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="28" customHeight="1">
+    <row r="19" spans="1:12" ht="28" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
@@ -4223,16 +4367,16 @@
         <v>2028</v>
       </c>
       <c r="C19" s="5">
-        <v>4574320.44</v>
+        <v>4414320.44</v>
       </c>
       <c r="D19" s="5">
-        <v>10999320.44</v>
+        <v>10839320.44</v>
       </c>
       <c r="E19" s="5">
         <v>0</v>
       </c>
       <c r="F19" s="5">
-        <v>10999320.44</v>
+        <v>10839320.44</v>
       </c>
       <c r="G19" s="5">
         <v>5309917.36</v>
@@ -4241,11 +4385,20 @@
         <v>2029</v>
       </c>
       <c r="I19" s="5">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5">
+        <v>250</v>
+      </c>
+      <c r="K19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="5">
         <f>ROUND(F19-D19+E19,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="28" customHeight="1">
+    <row r="20" spans="1:12" ht="28" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>29</v>
       </c>
@@ -4256,26 +4409,35 @@
         <v>4552730.98</v>
       </c>
       <c r="D20" s="5">
-        <v>6136685.04</v>
+        <v>6215918.73</v>
       </c>
       <c r="E20" s="5">
         <v>0</v>
       </c>
       <c r="F20" s="5">
-        <v>6136685.04</v>
+        <v>6215918.73</v>
       </c>
       <c r="G20" s="5">
-        <v>1190048.13</v>
+        <v>1249577.57</v>
       </c>
       <c r="H20" s="6">
         <v>2029</v>
       </c>
       <c r="I20" s="5">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5">
+        <v>250</v>
+      </c>
+      <c r="K20" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="5">
         <f>ROUND(F20-D20+E20,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28" customHeight="1">
+    <row r="21" spans="1:12" ht="28" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>29</v>
       </c>
@@ -4286,26 +4448,35 @@
         <v>4696705.34</v>
       </c>
       <c r="D21" s="5">
-        <v>5653542.15</v>
+        <v>5774184.22</v>
       </c>
       <c r="E21" s="5">
         <v>0</v>
       </c>
       <c r="F21" s="5">
-        <v>5653542.15</v>
+        <v>5774184.22</v>
       </c>
       <c r="G21" s="5">
-        <v>653532.41</v>
+        <v>735932.5699999999</v>
       </c>
       <c r="H21" s="6">
         <v>2029</v>
       </c>
       <c r="I21" s="5">
+        <v>0</v>
+      </c>
+      <c r="J21" s="5">
+        <v>250</v>
+      </c>
+      <c r="K21" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="5">
         <f>ROUND(F21-D21+E21,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28" customHeight="1">
+    <row r="22" spans="1:12" ht="28" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>29</v>
       </c>
@@ -4313,29 +4484,38 @@
         <v>2031</v>
       </c>
       <c r="C22" s="5">
-        <v>8086742.37</v>
+        <v>8250794.2</v>
       </c>
       <c r="D22" s="5">
-        <v>9033252.91</v>
+        <v>9362312.99</v>
       </c>
       <c r="E22" s="5">
         <v>0</v>
       </c>
       <c r="F22" s="5">
-        <v>9033252.91</v>
+        <v>9362312.99</v>
       </c>
       <c r="G22" s="5">
-        <v>587708.5699999999</v>
+        <v>690165.72</v>
       </c>
       <c r="H22" s="6">
         <v>2029</v>
       </c>
       <c r="I22" s="5">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5">
+        <v>250</v>
+      </c>
+      <c r="K22" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="5">
         <f>ROUND(F22-D22+E22,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="28" customHeight="1">
+    <row r="23" spans="1:12" ht="28" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>29</v>
       </c>
@@ -4343,29 +4523,38 @@
         <v>2032</v>
       </c>
       <c r="C23" s="5">
-        <v>5167612.99</v>
+        <v>5007612.99</v>
       </c>
       <c r="D23" s="5">
-        <v>6105011.71</v>
+        <v>6152477.35</v>
       </c>
       <c r="E23" s="5">
         <v>0</v>
       </c>
       <c r="F23" s="5">
-        <v>6105011.71</v>
+        <v>6152477.35</v>
       </c>
       <c r="G23" s="5">
-        <v>529137.14</v>
+        <v>646246.08</v>
       </c>
       <c r="H23" s="6">
         <v>2029</v>
       </c>
       <c r="I23" s="5">
+        <v>0</v>
+      </c>
+      <c r="J23" s="5">
+        <v>250</v>
+      </c>
+      <c r="K23" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="5">
         <f>ROUND(F23-D23+E23,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="28" customHeight="1">
+    <row r="24" spans="1:12" ht="28" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>29</v>
       </c>
@@ -4373,29 +4562,38 @@
         <v>2033</v>
       </c>
       <c r="C24" s="5">
-        <v>5171800.07</v>
+        <v>5176098.66</v>
       </c>
       <c r="D24" s="5">
-        <v>6090622.45</v>
+        <v>6348028.86</v>
       </c>
       <c r="E24" s="5">
         <v>0</v>
       </c>
       <c r="F24" s="5">
-        <v>6090622.45</v>
+        <v>6348028.86</v>
       </c>
       <c r="G24" s="5">
-        <v>471501.16</v>
+        <v>601385.5</v>
       </c>
       <c r="H24" s="6">
         <v>2029</v>
       </c>
       <c r="I24" s="5">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <v>250</v>
+      </c>
+      <c r="K24" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="5">
         <f>ROUND(F24-D24+E24,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="28" customHeight="1">
+    <row r="25" spans="1:12" ht="28" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>29</v>
       </c>
@@ -4403,29 +4601,38 @@
         <v>2034</v>
       </c>
       <c r="C25" s="5">
-        <v>5508635.21</v>
+        <v>5348635.21</v>
       </c>
       <c r="D25" s="5">
-        <v>6417698.03</v>
+        <v>7055723.32</v>
       </c>
       <c r="E25" s="5">
         <v>0</v>
       </c>
       <c r="F25" s="5">
-        <v>6417698.03</v>
+        <v>7055723.32</v>
       </c>
       <c r="G25" s="5">
-        <v>424084.52</v>
+        <v>796369.2</v>
       </c>
       <c r="H25" s="6">
         <v>2029</v>
       </c>
       <c r="I25" s="5">
+        <v>500000</v>
+      </c>
+      <c r="J25" s="5">
+        <v>250</v>
+      </c>
+      <c r="K25" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="5">
         <f>ROUND(F25-D25+E25,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="28" customHeight="1">
+    <row r="26" spans="1:12" ht="28" customHeight="1">
       <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
@@ -4433,29 +4640,38 @@
         <v>2035</v>
       </c>
       <c r="C26" s="5">
-        <v>8810416.41</v>
+        <v>8974976.779999999</v>
       </c>
       <c r="D26" s="5">
-        <v>9707856.93</v>
+        <v>10220208.39</v>
       </c>
       <c r="E26" s="5">
         <v>0</v>
       </c>
       <c r="F26" s="5">
-        <v>9707856.93</v>
+        <v>10220208.39</v>
       </c>
       <c r="G26" s="5">
-        <v>380602.39</v>
+        <v>528099.76</v>
       </c>
       <c r="H26" s="6">
         <v>2029</v>
       </c>
       <c r="I26" s="5">
+        <v>0</v>
+      </c>
+      <c r="J26" s="5">
+        <v>250</v>
+      </c>
+      <c r="K26" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="5">
         <f>ROUND(F26-D26+E26,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="28" customHeight="1">
+    <row r="27" spans="1:12" ht="28" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>29</v>
       </c>
@@ -4463,29 +4679,38 @@
         <v>2036</v>
       </c>
       <c r="C27" s="5">
-        <v>5887384.33</v>
+        <v>5892081.51</v>
       </c>
       <c r="D27" s="5">
-        <v>7024378.11</v>
+        <v>7426658.86</v>
       </c>
       <c r="E27" s="5">
         <v>0</v>
       </c>
       <c r="F27" s="5">
-        <v>7024378.11</v>
+        <v>7426658.86</v>
       </c>
       <c r="G27" s="5">
-        <v>438360.32</v>
+        <v>591646</v>
       </c>
       <c r="H27" s="6">
         <v>2029</v>
       </c>
       <c r="I27" s="5">
+        <v>0</v>
+      </c>
+      <c r="J27" s="5">
+        <v>250</v>
+      </c>
+      <c r="K27" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="5">
         <f>ROUND(F27-D27+E27,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="28" customHeight="1">
+    <row r="28" spans="1:12" ht="28" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>30</v>
       </c>
@@ -4511,11 +4736,20 @@
         <v>2029</v>
       </c>
       <c r="I28" s="5">
+        <v>0</v>
+      </c>
+      <c r="J28" s="5">
+        <v>250</v>
+      </c>
+      <c r="K28" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="5">
         <f>ROUND(F28-D28+E28,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="28" customHeight="1">
+    <row r="29" spans="1:12" ht="28" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>30</v>
       </c>
@@ -4541,11 +4775,20 @@
         <v>2029</v>
       </c>
       <c r="I29" s="5">
+        <v>0</v>
+      </c>
+      <c r="J29" s="5">
+        <v>250</v>
+      </c>
+      <c r="K29" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" s="5">
         <f>ROUND(F29-D29+E29,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="28" customHeight="1">
+    <row r="30" spans="1:12" ht="28" customHeight="1">
       <c r="A30" s="4" t="s">
         <v>30</v>
       </c>
@@ -4553,16 +4796,16 @@
         <v>2028</v>
       </c>
       <c r="C30" s="5">
-        <v>6056718.9</v>
+        <v>6220426.9</v>
       </c>
       <c r="D30" s="5">
-        <v>12481718.9</v>
+        <v>12645426.9</v>
       </c>
       <c r="E30" s="5">
         <v>0</v>
       </c>
       <c r="F30" s="5">
-        <v>12481718.9</v>
+        <v>12645426.9</v>
       </c>
       <c r="G30" s="5">
         <v>5309917.36</v>
@@ -4571,11 +4814,20 @@
         <v>2029</v>
       </c>
       <c r="I30" s="5">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5">
+        <v>250</v>
+      </c>
+      <c r="K30" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" s="5">
         <f>ROUND(F30-D30+E30,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="28" customHeight="1">
+    <row r="31" spans="1:12" ht="28" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
@@ -4583,29 +4835,38 @@
         <v>2029</v>
       </c>
       <c r="C31" s="5">
-        <v>6769362.73</v>
+        <v>6609362.73</v>
       </c>
       <c r="D31" s="5">
-        <v>8200504.13</v>
+        <v>8127391.34</v>
       </c>
       <c r="E31" s="5">
         <v>0</v>
       </c>
       <c r="F31" s="5">
-        <v>8200504.13</v>
+        <v>8127391.34</v>
       </c>
       <c r="G31" s="5">
-        <v>1075237.72</v>
+        <v>1140517.36</v>
       </c>
       <c r="H31" s="6">
         <v>2029</v>
       </c>
       <c r="I31" s="5">
+        <v>0</v>
+      </c>
+      <c r="J31" s="5">
+        <v>250</v>
+      </c>
+      <c r="K31" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" s="5">
         <f>ROUND(F31-D31+E31,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="28" customHeight="1">
+    <row r="32" spans="1:12" ht="28" customHeight="1">
       <c r="A32" s="4" t="s">
         <v>30</v>
       </c>
@@ -4613,29 +4874,38 @@
         <v>2030</v>
       </c>
       <c r="C32" s="5">
-        <v>7319367.57</v>
+        <v>7483301.39</v>
       </c>
       <c r="D32" s="5">
-        <v>7644450.82</v>
+        <v>7946585.77</v>
       </c>
       <c r="E32" s="5">
         <v>0</v>
       </c>
       <c r="F32" s="5">
-        <v>7644450.82</v>
+        <v>7946585.77</v>
       </c>
       <c r="G32" s="5">
-        <v>222036.23</v>
+        <v>316429.47</v>
       </c>
       <c r="H32" s="6">
         <v>2029</v>
       </c>
       <c r="I32" s="5">
+        <v>0</v>
+      </c>
+      <c r="J32" s="5">
+        <v>250</v>
+      </c>
+      <c r="K32" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" s="5">
         <f>ROUND(F32-D32+E32,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="28" customHeight="1">
+    <row r="33" spans="1:12" ht="28" customHeight="1">
       <c r="A33" s="4" t="s">
         <v>30</v>
       </c>
@@ -4643,29 +4913,38 @@
         <v>2031</v>
       </c>
       <c r="C33" s="5">
-        <v>18913517.47</v>
+        <v>19077569.31</v>
       </c>
       <c r="D33" s="5">
-        <v>18904517.18</v>
+        <v>22261976.59</v>
       </c>
       <c r="E33" s="5">
         <v>0</v>
       </c>
       <c r="F33" s="5">
-        <v>18904517.18</v>
+        <v>22261976.59</v>
       </c>
       <c r="G33" s="5">
-        <v>-5588.47</v>
+        <v>1977266.38</v>
       </c>
       <c r="H33" s="6">
         <v>2029</v>
       </c>
       <c r="I33" s="5">
+        <v>3000000</v>
+      </c>
+      <c r="J33" s="5">
+        <v>500</v>
+      </c>
+      <c r="K33" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L33" s="5">
         <f>ROUND(F33-D33+E33,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="28" customHeight="1">
+    <row r="34" spans="1:12" ht="28" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>30</v>
       </c>
@@ -4673,29 +4952,38 @@
         <v>2032</v>
       </c>
       <c r="C34" s="5">
-        <v>9371803.73</v>
+        <v>9375977.119999999</v>
       </c>
       <c r="D34" s="5">
-        <v>9136446.050000001</v>
+        <v>9395711.710000001</v>
       </c>
       <c r="E34" s="5">
         <v>0</v>
       </c>
       <c r="F34" s="5">
-        <v>9136446.050000001</v>
+        <v>9395711.710000001</v>
       </c>
       <c r="G34" s="5">
-        <v>-132853.27</v>
+        <v>11139.66</v>
       </c>
       <c r="H34" s="6">
         <v>2029</v>
       </c>
       <c r="I34" s="5">
+        <v>0</v>
+      </c>
+      <c r="J34" s="5">
+        <v>500</v>
+      </c>
+      <c r="K34" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L34" s="5">
         <f>ROUND(F34-D34+E34,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="28" customHeight="1">
+    <row r="35" spans="1:12" ht="28" customHeight="1">
       <c r="A35" s="4" t="s">
         <v>30</v>
       </c>
@@ -4703,29 +4991,38 @@
         <v>2033</v>
       </c>
       <c r="C35" s="5">
-        <v>10974029.64</v>
+        <v>11142626.82</v>
       </c>
       <c r="D35" s="5">
-        <v>10268437.64</v>
+        <v>10766011.76</v>
       </c>
       <c r="E35" s="5">
         <v>0</v>
       </c>
       <c r="F35" s="5">
-        <v>10268437.64</v>
+        <v>10766011.76</v>
       </c>
       <c r="G35" s="5">
-        <v>-362080.26</v>
+        <v>-193263.08</v>
       </c>
       <c r="H35" s="6">
         <v>2029</v>
       </c>
       <c r="I35" s="5">
+        <v>0</v>
+      </c>
+      <c r="J35" s="5">
+        <v>500</v>
+      </c>
+      <c r="K35" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L35" s="5">
         <f>ROUND(F35-D35+E35,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="28" customHeight="1">
+    <row r="36" spans="1:12" ht="28" customHeight="1">
       <c r="A36" s="4" t="s">
         <v>30</v>
       </c>
@@ -4733,29 +5030,38 @@
         <v>2034</v>
       </c>
       <c r="C36" s="5">
-        <v>12483602.75</v>
+        <v>12328030.3</v>
       </c>
       <c r="D36" s="5">
-        <v>11292123.78</v>
+        <v>12047294.88</v>
       </c>
       <c r="E36" s="5">
         <v>0</v>
       </c>
       <c r="F36" s="5">
-        <v>11292123.78</v>
+        <v>12047294.88</v>
       </c>
       <c r="G36" s="5">
-        <v>-555833.73</v>
+        <v>-130965.15</v>
       </c>
       <c r="H36" s="6">
         <v>2029</v>
       </c>
       <c r="I36" s="5">
+        <v>500000</v>
+      </c>
+      <c r="J36" s="5">
+        <v>500</v>
+      </c>
+      <c r="K36" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L36" s="5">
         <f>ROUND(F36-D36+E36,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="28" customHeight="1">
+    <row r="37" spans="1:12" ht="28" customHeight="1">
       <c r="A37" s="4" t="s">
         <v>30</v>
       </c>
@@ -4763,29 +5069,38 @@
         <v>2035</v>
       </c>
       <c r="C37" s="5">
-        <v>38138502.54</v>
+        <v>38467623.29</v>
       </c>
       <c r="D37" s="5">
-        <v>36191624.61</v>
+        <v>37034254.5</v>
       </c>
       <c r="E37" s="5">
         <v>0</v>
       </c>
       <c r="F37" s="5">
-        <v>36191624.61</v>
+        <v>37034254.5</v>
       </c>
       <c r="G37" s="5">
-        <v>-825666.29</v>
+        <v>-607888.29</v>
       </c>
       <c r="H37" s="6">
         <v>2029</v>
       </c>
       <c r="I37" s="5">
+        <v>0</v>
+      </c>
+      <c r="J37" s="5">
+        <v>500</v>
+      </c>
+      <c r="K37" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L37" s="5">
         <f>ROUND(F37-D37+E37,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="28" customHeight="1">
+    <row r="38" spans="1:12" ht="28" customHeight="1">
       <c r="A38" s="4" t="s">
         <v>30</v>
       </c>
@@ -4793,29 +5108,38 @@
         <v>2036</v>
       </c>
       <c r="C38" s="5">
-        <v>17148603.13</v>
+        <v>17157997.5</v>
       </c>
       <c r="D38" s="5">
-        <v>14670842.94</v>
+        <v>15314266.78</v>
       </c>
       <c r="E38" s="5">
         <v>0</v>
       </c>
       <c r="F38" s="5">
-        <v>14670842.94</v>
+        <v>15314266.78</v>
       </c>
       <c r="G38" s="5">
-        <v>-955283.8100000001</v>
+        <v>-710838.01</v>
       </c>
       <c r="H38" s="6">
         <v>2029</v>
       </c>
       <c r="I38" s="5">
+        <v>0</v>
+      </c>
+      <c r="J38" s="5">
+        <v>500</v>
+      </c>
+      <c r="K38" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L38" s="5">
         <f>ROUND(F38-D38+E38,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="28" customHeight="1">
+    <row r="39" spans="1:12" ht="28" customHeight="1">
       <c r="A39" s="4" t="s">
         <v>31</v>
       </c>
@@ -4841,11 +5165,20 @@
         <v>2031</v>
       </c>
       <c r="I39" s="5">
+        <v>0</v>
+      </c>
+      <c r="J39" s="5">
+        <v>250</v>
+      </c>
+      <c r="K39" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L39" s="5">
         <f>ROUND(F39-D39+E39,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="28" customHeight="1">
+    <row r="40" spans="1:12" ht="28" customHeight="1">
       <c r="A40" s="4" t="s">
         <v>31</v>
       </c>
@@ -4871,11 +5204,20 @@
         <v>2031</v>
       </c>
       <c r="I40" s="5">
+        <v>0</v>
+      </c>
+      <c r="J40" s="5">
+        <v>250</v>
+      </c>
+      <c r="K40" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L40" s="5">
         <f>ROUND(F40-D40+E40,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="28" customHeight="1">
+    <row r="41" spans="1:12" ht="28" customHeight="1">
       <c r="A41" s="4" t="s">
         <v>31</v>
       </c>
@@ -4883,16 +5225,16 @@
         <v>2028</v>
       </c>
       <c r="C41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="D41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="E41" s="5">
         <v>0</v>
       </c>
       <c r="F41" s="5">
-        <v>5228516.2</v>
+        <v>5392224.2</v>
       </c>
       <c r="G41" s="5">
         <v>0</v>
@@ -4901,11 +5243,20 @@
         <v>2031</v>
       </c>
       <c r="I41" s="5">
+        <v>0</v>
+      </c>
+      <c r="J41" s="5">
+        <v>250</v>
+      </c>
+      <c r="K41" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" s="5">
         <f>ROUND(F41-D41+E41,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="28" customHeight="1">
+    <row r="42" spans="1:12" ht="28" customHeight="1">
       <c r="A42" s="4" t="s">
         <v>31</v>
       </c>
@@ -4913,16 +5264,16 @@
         <v>2029</v>
       </c>
       <c r="C42" s="5">
-        <v>5262359.14</v>
+        <v>5102359.14</v>
       </c>
       <c r="D42" s="5">
-        <v>9637359.140000001</v>
+        <v>9477359.140000001</v>
       </c>
       <c r="E42" s="5">
         <v>0</v>
       </c>
       <c r="F42" s="5">
-        <v>9637359.140000001</v>
+        <v>9477359.140000001</v>
       </c>
       <c r="G42" s="5">
         <v>3287002.25</v>
@@ -4931,11 +5282,20 @@
         <v>2031</v>
       </c>
       <c r="I42" s="5">
+        <v>0</v>
+      </c>
+      <c r="J42" s="5">
+        <v>250</v>
+      </c>
+      <c r="K42" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L42" s="5">
         <f>ROUND(F42-D42+E42,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="28" customHeight="1">
+    <row r="43" spans="1:12" ht="28" customHeight="1">
       <c r="A43" s="4" t="s">
         <v>31</v>
       </c>
@@ -4943,16 +5303,16 @@
         <v>2030</v>
       </c>
       <c r="C43" s="5">
-        <v>5283350.63</v>
+        <v>5447284.45</v>
       </c>
       <c r="D43" s="5">
-        <v>11708350.63</v>
+        <v>11872284.45</v>
       </c>
       <c r="E43" s="5">
         <v>0</v>
       </c>
       <c r="F43" s="5">
-        <v>11708350.63</v>
+        <v>11872284.45</v>
       </c>
       <c r="G43" s="5">
         <v>4388361.45</v>
@@ -4961,11 +5321,20 @@
         <v>2031</v>
       </c>
       <c r="I43" s="5">
+        <v>0</v>
+      </c>
+      <c r="J43" s="5">
+        <v>250</v>
+      </c>
+      <c r="K43" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" s="5">
         <f>ROUND(F43-D43+E43,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="28" customHeight="1">
+    <row r="44" spans="1:12" ht="28" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>31</v>
       </c>
@@ -4976,26 +5345,35 @@
         <v>11370189.81</v>
       </c>
       <c r="D44" s="5">
-        <v>12831404.33</v>
+        <v>13002817.97</v>
       </c>
       <c r="E44" s="5">
         <v>0</v>
       </c>
       <c r="F44" s="5">
-        <v>12831404.33</v>
+        <v>13002817.97</v>
       </c>
       <c r="G44" s="5">
-        <v>907299.26</v>
+        <v>1013733.64</v>
       </c>
       <c r="H44" s="6">
         <v>2031</v>
       </c>
       <c r="I44" s="5">
+        <v>0</v>
+      </c>
+      <c r="J44" s="5">
+        <v>250</v>
+      </c>
+      <c r="K44" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" s="5">
         <f>ROUND(F44-D44+E44,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="28" customHeight="1">
+    <row r="45" spans="1:12" ht="28" customHeight="1">
       <c r="A45" s="4" t="s">
         <v>31</v>
       </c>
@@ -5003,29 +5381,38 @@
         <v>2032</v>
       </c>
       <c r="C45" s="5">
-        <v>5722998.42</v>
+        <v>5887171.81</v>
       </c>
       <c r="D45" s="5">
-        <v>6366026.75</v>
+        <v>6750709.55</v>
       </c>
       <c r="E45" s="5">
         <v>0</v>
       </c>
       <c r="F45" s="5">
-        <v>6366026.75</v>
+        <v>6750709.55</v>
       </c>
       <c r="G45" s="5">
-        <v>362972.73</v>
+        <v>487444.54</v>
       </c>
       <c r="H45" s="6">
         <v>2031</v>
       </c>
       <c r="I45" s="5">
+        <v>0</v>
+      </c>
+      <c r="J45" s="5">
+        <v>250</v>
+      </c>
+      <c r="K45" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L45" s="5">
         <f>ROUND(F45-D45+E45,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="28" customHeight="1">
+    <row r="46" spans="1:12" ht="28" customHeight="1">
       <c r="A46" s="4" t="s">
         <v>31</v>
       </c>
@@ -5033,29 +5420,38 @@
         <v>2033</v>
       </c>
       <c r="C46" s="5">
-        <v>6073851.46</v>
+        <v>6203525.54</v>
       </c>
       <c r="D46" s="5">
-        <v>6704114.95</v>
+        <v>6978514.05</v>
       </c>
       <c r="E46" s="5">
         <v>0</v>
       </c>
       <c r="F46" s="5">
-        <v>6704114.95</v>
+        <v>6978514.05</v>
       </c>
       <c r="G46" s="5">
-        <v>323424.83</v>
+        <v>397691.65</v>
       </c>
       <c r="H46" s="6">
         <v>2031</v>
       </c>
       <c r="I46" s="5">
+        <v>0</v>
+      </c>
+      <c r="J46" s="5">
+        <v>250</v>
+      </c>
+      <c r="K46" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" s="5">
         <f>ROUND(F46-D46+E46,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="28" customHeight="1">
+    <row r="47" spans="1:12" ht="28" customHeight="1">
       <c r="A47" s="4" t="s">
         <v>31</v>
       </c>
@@ -5063,29 +5459,38 @@
         <v>2034</v>
       </c>
       <c r="C47" s="5">
-        <v>6711178.62</v>
+        <v>6715606.16</v>
       </c>
       <c r="D47" s="5">
-        <v>7206504.41</v>
+        <v>8034465.18</v>
       </c>
       <c r="E47" s="5">
         <v>0</v>
       </c>
       <c r="F47" s="5">
-        <v>7206504.41</v>
+        <v>8034465.18</v>
       </c>
       <c r="G47" s="5">
-        <v>231073.14</v>
+        <v>615257.47</v>
       </c>
       <c r="H47" s="6">
         <v>2031</v>
       </c>
       <c r="I47" s="5">
+        <v>500000</v>
+      </c>
+      <c r="J47" s="5">
+        <v>250</v>
+      </c>
+      <c r="K47" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L47" s="5">
         <f>ROUND(F47-D47+E47,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="28" customHeight="1">
+    <row r="48" spans="1:12" ht="28" customHeight="1">
       <c r="A48" s="4" t="s">
         <v>31</v>
       </c>
@@ -5093,29 +5498,38 @@
         <v>2035</v>
       </c>
       <c r="C48" s="5">
-        <v>14327304.3</v>
+        <v>14491864.67</v>
       </c>
       <c r="D48" s="5">
-        <v>14671645.95</v>
+        <v>15213863.77</v>
       </c>
       <c r="E48" s="5">
         <v>0</v>
       </c>
       <c r="F48" s="5">
-        <v>14671645.95</v>
+        <v>15213863.77</v>
       </c>
       <c r="G48" s="5">
-        <v>146034.47</v>
+        <v>306198.1</v>
       </c>
       <c r="H48" s="6">
         <v>2031</v>
       </c>
       <c r="I48" s="5">
+        <v>0</v>
+      </c>
+      <c r="J48" s="5">
+        <v>250</v>
+      </c>
+      <c r="K48" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L48" s="5">
         <f>ROUND(F48-D48+E48,2)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="28" customHeight="1">
+    <row r="49" spans="1:12" ht="28" customHeight="1">
       <c r="A49" s="4" t="s">
         <v>31</v>
       </c>
@@ -5123,33 +5537,42 @@
         <v>2036</v>
       </c>
       <c r="C49" s="5">
-        <v>7604996.94</v>
+        <v>7774391.31</v>
       </c>
       <c r="D49" s="5">
-        <v>8184868.53</v>
+        <v>8792810.789999999</v>
       </c>
       <c r="E49" s="5">
         <v>0</v>
       </c>
       <c r="F49" s="5">
-        <v>8184868.53</v>
+        <v>8792810.789999999</v>
       </c>
       <c r="G49" s="5">
-        <v>223565.6</v>
+        <v>392644.8</v>
       </c>
       <c r="H49" s="6">
         <v>2031</v>
       </c>
       <c r="I49" s="5">
+        <v>0</v>
+      </c>
+      <c r="J49" s="5">
+        <v>250</v>
+      </c>
+      <c r="K49" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L49" s="5">
         <f>ROUND(F49-D49+E49,2)</f>
         <v>0.0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H49"/>
+  <autoFilter ref="A5:K49"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="landscape"/>
@@ -5173,7 +5596,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5198,19 +5621,19 @@
     </row>
     <row r="5" spans="1:6" ht="36" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>26</v>
@@ -5218,10 +5641,10 @@
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C6" s="5">
         <v>3</v>
@@ -5239,10 +5662,10 @@
     </row>
     <row r="7" spans="1:6" ht="28" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C7" s="5">
         <v>2</v>
@@ -5260,10 +5683,10 @@
     </row>
     <row r="8" spans="1:6" ht="28" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C8" s="5">
         <v>2</v>
@@ -5281,10 +5704,10 @@
     </row>
     <row r="9" spans="1:6" ht="28" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C9" s="5">
         <v>3</v>
@@ -5302,10 +5725,10 @@
     </row>
     <row r="10" spans="1:6" ht="28" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C10" s="5">
         <v>2</v>
@@ -5323,10 +5746,10 @@
     </row>
     <row r="11" spans="1:6" ht="28" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C11" s="5">
         <v>2</v>
@@ -5344,10 +5767,10 @@
     </row>
     <row r="12" spans="1:6" ht="28" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C12" s="5">
         <v>2</v>
@@ -5365,10 +5788,10 @@
     </row>
     <row r="13" spans="1:6" ht="28" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -5386,10 +5809,10 @@
     </row>
     <row r="14" spans="1:6" ht="28" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C14" s="5">
         <v>2</v>
@@ -5407,10 +5830,10 @@
     </row>
     <row r="15" spans="1:6" ht="28" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
@@ -5456,7 +5879,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5487,25 +5910,25 @@
     </row>
     <row r="5" spans="1:8" ht="36" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>26</v>
@@ -5513,22 +5936,22 @@
     </row>
     <row r="6" spans="1:8" ht="28" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D6" s="5">
         <v>3000000</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G6" s="5">
         <v>0</v>
@@ -5540,19 +5963,19 @@
     </row>
     <row r="7" spans="1:8" ht="28" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D7" s="5">
         <v>200000</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="5">
@@ -5565,19 +5988,19 @@
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D8" s="5">
         <v>300000</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="5">
@@ -5590,19 +6013,19 @@
     </row>
     <row r="9" spans="1:8" ht="28" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D9" s="5">
         <v>700000</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="5">
@@ -5615,19 +6038,19 @@
     </row>
     <row r="10" spans="1:8" ht="28" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D10" s="5">
         <v>1000000</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="5">
@@ -5640,19 +6063,19 @@
     </row>
     <row r="11" spans="1:8" ht="28" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D11" s="5">
         <v>3500000</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="5">
@@ -5665,19 +6088,19 @@
     </row>
     <row r="12" spans="1:8" ht="28" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D12" s="5">
         <v>1000000</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="5">
@@ -5690,19 +6113,19 @@
     </row>
     <row r="13" spans="1:8" ht="28" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D13" s="5">
         <v>5000000</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="5">
@@ -5715,19 +6138,19 @@
     </row>
     <row r="14" spans="1:8" ht="28" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D14" s="5">
         <v>300000</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="5">
@@ -5740,19 +6163,19 @@
     </row>
     <row r="15" spans="1:8" ht="28" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="D15" s="5">
         <v>500000</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="5">
@@ -5791,7 +6214,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5828,19 +6251,19 @@
         <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>26</v>
@@ -5908,16 +6331,16 @@
         <v>2028</v>
       </c>
       <c r="C8" s="5">
-        <v>232372162.6662</v>
+        <v>232495495.9999</v>
       </c>
       <c r="D8" s="5">
-        <v>101845775.7197</v>
+        <v>102009483.7197</v>
       </c>
       <c r="E8" s="5">
-        <v>130526386.9465</v>
+        <v>130486012.2802</v>
       </c>
       <c r="F8" s="5">
-        <v>-6156782.5559</v>
+        <v>-6197157.2222</v>
       </c>
       <c r="G8" s="5">
         <v>11683039</v>
@@ -5935,16 +6358,16 @@
         <v>2029</v>
       </c>
       <c r="C9" s="5">
-        <v>244543785.2153</v>
+        <v>244503785.2157</v>
       </c>
       <c r="D9" s="5">
         <v>103120591.1948</v>
       </c>
       <c r="E9" s="5">
-        <v>141423194.0205</v>
+        <v>141383194.0209</v>
       </c>
       <c r="F9" s="5">
-        <v>2954851.2775</v>
+        <v>2951517.9442</v>
       </c>
       <c r="G9" s="5">
         <v>26897283.856</v>
@@ -5962,19 +6385,19 @@
         <v>2030</v>
       </c>
       <c r="C10" s="5">
-        <v>257058705.3438</v>
+        <v>256978104.8607</v>
       </c>
       <c r="D10" s="5">
         <v>102839746.4188</v>
       </c>
       <c r="E10" s="5">
-        <v>154218958.925</v>
+        <v>154138358.4419</v>
       </c>
       <c r="F10" s="5">
-        <v>12795764.9045</v>
+        <v>12755164.421</v>
       </c>
       <c r="G10" s="5">
-        <v>44643430.176</v>
+        <v>44479496.3588</v>
       </c>
       <c r="H10" s="5">
         <f>ROUND(C10-D10-E10,2)</f>
@@ -5989,19 +6412,19 @@
         <v>2031</v>
       </c>
       <c r="C11" s="5">
-        <v>274210236.9065</v>
+        <v>274089636.4227</v>
       </c>
       <c r="D11" s="5">
         <v>101874826.9716</v>
       </c>
       <c r="E11" s="5">
-        <v>172335409.9349</v>
+        <v>172214809.4511</v>
       </c>
       <c r="F11" s="5">
-        <v>18116451.0099</v>
+        <v>18076451.0092</v>
       </c>
       <c r="G11" s="5">
-        <v>59806731.4704</v>
+        <v>59642797.6532</v>
       </c>
       <c r="H11" s="5">
         <f>ROUND(C11-D11-E11,2)</f>
@@ -6010,7 +6433,7 @@
     </row>
     <row r="12" spans="1:8" ht="28" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B12" s="6">
         <v>2026</v>
@@ -6037,22 +6460,22 @@
     </row>
     <row r="13" spans="1:8" ht="28" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B13" s="6">
         <v>2027</v>
       </c>
       <c r="C13" s="5">
-        <v>222547911.9141</v>
+        <v>222671245.2478</v>
       </c>
       <c r="D13" s="5">
-        <v>127566316.5225</v>
+        <v>127729916.5225</v>
       </c>
       <c r="E13" s="5">
-        <v>94981595.3916</v>
+        <v>94941328.7253</v>
       </c>
       <c r="F13" s="5">
-        <v>-43464469.8083</v>
+        <v>-43504736.4746</v>
       </c>
       <c r="G13" s="5">
         <v>7751200</v>
@@ -6064,46 +6487,46 @@
     </row>
     <row r="14" spans="1:8" ht="28" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B14" s="6">
         <v>2028</v>
       </c>
       <c r="C14" s="5">
-        <v>228774285.3086</v>
+        <v>228734285.309</v>
       </c>
       <c r="D14" s="5">
-        <v>161592572.3917</v>
+        <v>161596172.3917</v>
       </c>
       <c r="E14" s="5">
-        <v>67181712.91689999</v>
+        <v>67138112.9173</v>
       </c>
       <c r="F14" s="5">
-        <v>-44111011.4747</v>
+        <v>-44114344.808</v>
       </c>
       <c r="G14" s="5">
         <v>7356664</v>
       </c>
       <c r="H14" s="5">
         <f>ROUND(C14-D14-E14,2)</f>
-        <v>0.0</v>
+        <v>-0.0</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B15" s="6">
         <v>2029</v>
       </c>
       <c r="C15" s="5">
-        <v>225969600.5208</v>
+        <v>225929600.5212</v>
       </c>
       <c r="D15" s="5">
-        <v>183879099.2197</v>
+        <v>183882699.2197</v>
       </c>
       <c r="E15" s="5">
-        <v>42090501.3011</v>
+        <v>42046901.3015</v>
       </c>
       <c r="F15" s="5">
         <v>-40479996.6158</v>
@@ -6118,19 +6541,19 @@
     </row>
     <row r="16" spans="1:8" ht="28" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B16" s="6">
         <v>2030</v>
       </c>
       <c r="C16" s="5">
-        <v>226243459.4178</v>
+        <v>226203459.4182</v>
       </c>
       <c r="D16" s="5">
-        <v>195438527.3909</v>
+        <v>195442127.3909</v>
       </c>
       <c r="E16" s="5">
-        <v>30804932.0269</v>
+        <v>30761332.0273</v>
       </c>
       <c r="F16" s="5">
         <v>-34101849.2742</v>
@@ -6145,22 +6568,22 @@
     </row>
     <row r="17" spans="1:8" ht="28" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B17" s="6">
         <v>2031</v>
       </c>
       <c r="C17" s="5">
-        <v>225249158.3385</v>
+        <v>225369158.3389</v>
       </c>
       <c r="D17" s="5">
-        <v>199579450.1941</v>
+        <v>199747102.0253</v>
       </c>
       <c r="E17" s="5">
-        <v>25669708.1444</v>
+        <v>25622056.3136</v>
       </c>
       <c r="F17" s="5">
-        <v>-29160555.8825</v>
+        <v>-29164607.7137</v>
       </c>
       <c r="G17" s="5">
         <v>4834452</v>
@@ -6172,7 +6595,7 @@
     </row>
     <row r="18" spans="1:8" ht="28" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B18" s="6">
         <v>2026</v>
@@ -6199,7 +6622,7 @@
     </row>
     <row r="19" spans="1:8" ht="28" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B19" s="6">
         <v>2027</v>
@@ -6226,22 +6649,22 @@
     </row>
     <row r="20" spans="1:8" ht="28" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B20" s="6">
         <v>2028</v>
       </c>
       <c r="C20" s="5">
-        <v>248658014.2988</v>
+        <v>248781347.6325</v>
       </c>
       <c r="D20" s="5">
         <v>99230182.1356</v>
       </c>
       <c r="E20" s="5">
-        <v>149427832.1632</v>
+        <v>149551165.4969</v>
       </c>
       <c r="F20" s="5">
-        <v>-1108878.4257</v>
+        <v>-1149253.092</v>
       </c>
       <c r="G20" s="5">
         <v>9056450</v>
@@ -6253,22 +6676,22 @@
     </row>
     <row r="21" spans="1:8" ht="28" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B21" s="6">
         <v>2029</v>
       </c>
       <c r="C21" s="5">
-        <v>270778795.7575</v>
+        <v>270738795.7579</v>
       </c>
       <c r="D21" s="5">
         <v>105272642.4636</v>
       </c>
       <c r="E21" s="5">
-        <v>165506153.2939</v>
+        <v>165466153.2943</v>
       </c>
       <c r="F21" s="5">
-        <v>10193533.6254</v>
+        <v>10190200.2921</v>
       </c>
       <c r="G21" s="5">
         <v>29713487.2589</v>
@@ -6280,25 +6703,25 @@
     </row>
     <row r="22" spans="1:8" ht="28" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B22" s="6">
         <v>2030</v>
       </c>
       <c r="C22" s="5">
-        <v>293846026.1345</v>
+        <v>293765425.6514</v>
       </c>
       <c r="D22" s="5">
         <v>105392117.9243</v>
       </c>
       <c r="E22" s="5">
-        <v>188453908.2102</v>
+        <v>188373307.7271</v>
       </c>
       <c r="F22" s="5">
-        <v>22947754.9163</v>
+        <v>22907154.4328</v>
       </c>
       <c r="G22" s="5">
-        <v>55964511.4897</v>
+        <v>55800577.6725</v>
       </c>
       <c r="H22" s="5">
         <f>ROUND(C22-D22-E22,2)</f>
@@ -6307,25 +6730,25 @@
     </row>
     <row r="23" spans="1:8" ht="28" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B23" s="6">
         <v>2031</v>
       </c>
       <c r="C23" s="5">
-        <v>323529686.9231</v>
+        <v>323368367.9418</v>
       </c>
       <c r="D23" s="5">
         <v>104255265.0024</v>
       </c>
       <c r="E23" s="5">
-        <v>219274421.9207</v>
+        <v>219113102.9394</v>
       </c>
       <c r="F23" s="5">
-        <v>30820513.7105</v>
+        <v>30739795.2123</v>
       </c>
       <c r="G23" s="5">
-        <v>83963276.5213</v>
+        <v>83635290.87289999</v>
       </c>
       <c r="H23" s="5">
         <f>ROUND(C23-D23-E23,2)</f>

</xml_diff>